<commit_message>
ci: refresh reports + Excel + Tableau (2025-11-04 00:41 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -798,6 +798,51 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:41:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:41:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:41:41</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ci: refresh reports + Excel + Tableau (2025-11-04 00:42 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -843,6 +843,51 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:42:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:42:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:42:24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ci: refresh reports + Excel + Tableau (2025-11-04 00:43 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -888,6 +888,51 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:43:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:43:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2025-11-04 00:43:49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(artifacts): refresh PDF + KPI Excel (2025-11-04 07:22)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -933,6 +933,51 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2025-11-04 01:52 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2025-11-04 01:52 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2025-11-04 01:52 UTC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ci: refresh reports + Excel + Tableau (2025-11-04 02:26 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,13 +32,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000DDD8"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6FA"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,10 +62,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -401,13 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Last Refreshed (UTC): 2025-11-04 02:09:06 UTC</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Last Refreshed (UTC): 2025-11-04 02:26 UTC</t>
         </is>
       </c>
     </row>
@@ -470,6 +485,51 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>2025-11-04 02:09:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-11-04 02:26 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-11-04 02:26 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-11-04 02:26 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(conflicts): resolved Excel and PDF merge conflicts after rebase
- Kept latest versions from main branch for KPI_Snapshot and PDF report
- Merged origin/main changes cleanly
- Verified all artifact updates and background formatting consistency
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,13 +32,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000DDD8"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6FA"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,10 +62,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -401,13 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Last Refreshed (UTC): 2025-11-04 02:09:06 UTC</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Last Refreshed (UTC): 2025-11-04 02:27 UTC</t>
         </is>
       </c>
     </row>
@@ -470,6 +485,51 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>2025-11-04 02:09:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-11-04 02:27 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-11-04 02:27 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-11-04 02:27 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports + Excel + Tableau (2025-11-05 12:01 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -422,7 +422,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2025-11-04 02:27 UTC</t>
+          <t>Last Refreshed (UTC): 2025-11-05 12:01 UTC</t>
         </is>
       </c>
     </row>
@@ -530,6 +530,51 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>2025-11-04 02:27 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025-11-05 12:01 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-11-05 12:01 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025-11-05 12:01 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports + Excel + Tableau (2025-11-05 14:37 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/KPI_Snapshot.xlsx
+++ b/04_Excel/KPI_Snapshot.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -422,7 +422,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2025-11-05 12:01 UTC</t>
+          <t>Last Refreshed (UTC): 2025-11-05 14:37 UTC</t>
         </is>
       </c>
     </row>
@@ -575,6 +575,51 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>2025-11-05 12:01 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>10641558.95</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2025-11-05 14:37 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4338</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-11-05 14:37 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2453.102570308898</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2025-11-05 14:37 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>